<commit_message>
Remove workbook instruction blocks
</commit_message>
<xml_diff>
--- a/results/江右游日记_二十三日_步驟五_API配對.xlsx
+++ b/results/江右游日记_二十三日_步驟五_API配對.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步驟五｜二十三日經緯度來源" sheetId="1" r:id="R5a7e15f767af4d1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步驟五｜二十三日經緯度來源" sheetId="2" r:id="R95d613252e0649e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -52,8 +52,14 @@
       <x:color rgb="FF172033"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -80,6 +86,11 @@
         <x:fgColor rgb="FFFEF3C7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0369A1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -92,7 +103,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -149,6 +160,26 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -158,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Day23Step5CompactCoordinates" displayName="Day23Step5CompactCoordinates" ref="A7:F23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:F23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Day23Step5CompactCoordinates" displayName="Day23Step5CompactCoordinates" ref="A3:F19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:F19"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="序號"/>
     <x:tableColumn id="2" name="日期"/>
@@ -376,342 +407,306 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="31" t="str">
         <x:v>步驟五｜二十三日經緯度及資料來源｜精簡版</x:v>
       </x:c>
-      <x:c r="B1" s="4"/>
-      <x:c r="C1" s="4"/>
-      <x:c r="D1" s="4"/>
-      <x:c r="E1" s="4"/>
-      <x:c r="F1" s="4"/>
-    </x:row>
-    <x:row r="2" ht="21" customHeight="1">
-      <x:c r="A2" s="8" t="str">
-        <x:v>篩選結果｜16 筆</x:v>
-      </x:c>
-      <x:c r="B2" s="8"/>
-      <x:c r="C2" s="8"/>
-      <x:c r="D2" s="8"/>
-      <x:c r="E2" s="8"/>
-      <x:c r="F2" s="8"/>
-    </x:row>
-    <x:row r="3" ht="45" customHeight="1">
-      <x:c r="A3" s="12" t="str">
-        <x:v>精簡版步驟五：只保留地點識別、經度、緯度及統一資料來源。各資料 API 的查詢結果已合併在「資料來源」欄，不再分開顯示 API 欄位。空白經緯度代表本輪沒有可通過限制並可追溯的座標。</x:v>
-      </x:c>
-      <x:c r="B3" s="12"/>
-      <x:c r="C3" s="12"/>
-      <x:c r="D3" s="12"/>
-      <x:c r="E3" s="12"/>
-      <x:c r="F3" s="12"/>
-    </x:row>
-    <x:row r="4" ht="18.75" customHeight="1">
-      <x:c r="A4" s="16" t="str">
-        <x:v>Prompt｜本步驟獨立操作指令</x:v>
-      </x:c>
-      <x:c r="B4" s="16"/>
-      <x:c r="C4" s="16"/>
-      <x:c r="D4" s="16"/>
-      <x:c r="E4" s="16"/>
-      <x:c r="F4" s="16"/>
-    </x:row>
-    <x:row r="5" ht="61.5" customHeight="1">
-      <x:c r="A5" s="12" t="str">
-        <x:v>請在指定經緯度範圍內以 CHGIS/TGAZ、Wikidata、OpenStreetMap/Nominatim、Amap 及 Google Maps 交叉核查候選；只輸出序號、日期、地名、經度_WGS84、緯度_WGS84、資料來源。若沒有通過名稱、年代、行政區、地物類型及範圍限制的座標，經緯度留空，資料來源寫明查詢來源及未採用原因，不分開建立各 API 欄位。</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-    </x:row>
-    <x:row r="7" ht="31.5" customHeight="1">
-      <x:c r="A7" s="20" t="str">
+      <x:c r="B1" s="31"/>
+      <x:c r="C1" s="31"/>
+      <x:c r="D1" s="31"/>
+      <x:c r="E1" s="31"/>
+      <x:c r="F1" s="31"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+    </x:row>
+    <x:row r="3" ht="31.5" customHeight="1">
+      <x:c r="A3" s="34" t="str">
         <x:v>序號</x:v>
       </x:c>
-      <x:c r="B7" s="20" t="str">
+      <x:c r="B3" s="34" t="str">
         <x:v>日期</x:v>
       </x:c>
-      <x:c r="C7" s="20" t="str">
+      <x:c r="C3" s="34" t="str">
         <x:v>地名</x:v>
       </x:c>
-      <x:c r="D7" s="20" t="str">
+      <x:c r="D3" s="34" t="str">
         <x:v>經度_WGS84</x:v>
       </x:c>
-      <x:c r="E7" s="20" t="str">
+      <x:c r="E3" s="34" t="str">
         <x:v>緯度_WGS84</x:v>
       </x:c>
-      <x:c r="F7" s="20" t="str">
+      <x:c r="F3" s="34" t="str">
         <x:v>資料來源</x:v>
       </x:c>
     </x:row>
+    <x:row r="4" ht="43.5" customHeight="1">
+      <x:c r="A4" t="n">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>张真人墓</x:v>
+      </x:c>
+      <x:c r="D4"/>
+      <x:c r="E4"/>
+      <x:c r="F4" t="str">
+        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="43.5" customHeight="1">
+      <x:c r="A5" t="n">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>五面峰</x:v>
+      </x:c>
+      <x:c r="D5"/>
+      <x:c r="E5"/>
+      <x:c r="F5" t="str">
+        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="43.5" customHeight="1">
+      <x:c r="A6" t="n">
+        <x:v>191</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>五面峰</x:v>
+      </x:c>
+      <x:c r="D6"/>
+      <x:c r="E6"/>
+      <x:c r="F6" t="str">
+        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="43.5" customHeight="1">
+      <x:c r="A7" t="n">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>西华</x:v>
+      </x:c>
+      <x:c r="D7"/>
+      <x:c r="E7"/>
+      <x:c r="F7" t="str">
+        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；有原始候選，但未同時通過名稱、類型及限制範圍；不得採用其座標。</x:v>
+      </x:c>
+    </x:row>
     <x:row r="8" ht="43.5" customHeight="1">
-      <x:c r="A8" s="25" t="n">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="B8" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C8" s="25" t="str">
-        <x:v>张真人墓</x:v>
-      </x:c>
-      <x:c r="D8" s="25"/>
-      <x:c r="E8" s="25"/>
-      <x:c r="F8" s="25" t="str">
-        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
+      <x:c r="A8" t="n">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>西华</x:v>
+      </x:c>
+      <x:c r="D8"/>
+      <x:c r="E8"/>
+      <x:c r="F8" t="str">
+        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；有原始候選，但未同時通過名稱、類型及限制範圍；不得採用其座標。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="43.5" customHeight="1">
-      <x:c r="A9" s="25" t="n">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="B9" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C9" s="25" t="str">
-        <x:v>五面峰</x:v>
-      </x:c>
-      <x:c r="D9" s="25"/>
-      <x:c r="E9" s="25"/>
-      <x:c r="F9" s="25" t="str">
+      <x:c r="A9" t="n">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>小隐岩</x:v>
+      </x:c>
+      <x:c r="D9"/>
+      <x:c r="E9"/>
+      <x:c r="F9" t="str">
         <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43.5" customHeight="1">
-      <x:c r="A10" s="25" t="n">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="B10" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C10" s="25" t="str">
-        <x:v>五面峰</x:v>
-      </x:c>
-      <x:c r="D10" s="25"/>
-      <x:c r="E10" s="25"/>
-      <x:c r="F10" s="25" t="str">
+      <x:c r="A10" t="n">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>朝真宫</x:v>
+      </x:c>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+      <x:c r="F10" t="str">
         <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="43.5" customHeight="1">
-      <x:c r="A11" s="25" t="n">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="B11" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C11" s="25" t="str">
-        <x:v>西华</x:v>
-      </x:c>
-      <x:c r="D11" s="25"/>
-      <x:c r="E11" s="25"/>
-      <x:c r="F11" s="25" t="str">
+      <x:c r="A11" t="n">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>大霍岭</x:v>
+      </x:c>
+      <x:c r="D11"/>
+      <x:c r="E11"/>
+      <x:c r="F11" t="str">
+        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="43.5" customHeight="1">
+      <x:c r="A12" t="n">
+        <x:v>627</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>龙骨山</x:v>
+      </x:c>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12" t="str">
         <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；有原始候選，但未同時通過名稱、類型及限制範圍；不得採用其座標。</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="43.5" customHeight="1">
-      <x:c r="A12" s="25" t="n">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="B12" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C12" s="25" t="str">
-        <x:v>西华</x:v>
-      </x:c>
-      <x:c r="D12" s="25"/>
-      <x:c r="E12" s="25"/>
-      <x:c r="F12" s="25" t="str">
+    <x:row r="13" ht="43.5" customHeight="1">
+      <x:c r="A13" t="n">
+        <x:v>628</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>骨岭</x:v>
+      </x:c>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13" t="str">
         <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；有原始候選，但未同時通過名稱、類型及限制範圍；不得採用其座標。</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="43.5" customHeight="1">
-      <x:c r="A13" s="25" t="n">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="B13" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C13" s="25" t="str">
-        <x:v>小隐岩</x:v>
-      </x:c>
-      <x:c r="D13" s="25"/>
-      <x:c r="E13" s="25"/>
-      <x:c r="F13" s="25" t="str">
-        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
-      </x:c>
-    </x:row>
     <x:row r="14" ht="43.5" customHeight="1">
-      <x:c r="A14" s="25" t="n">
-        <x:v>212</x:v>
-      </x:c>
-      <x:c r="B14" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C14" s="25" t="str">
-        <x:v>朝真宫</x:v>
-      </x:c>
-      <x:c r="D14" s="25"/>
-      <x:c r="E14" s="25"/>
-      <x:c r="F14" s="25" t="str">
+      <x:c r="A14" t="n">
+        <x:v>629</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>幞头岭</x:v>
+      </x:c>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14" t="str">
         <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="43.5" customHeight="1">
-      <x:c r="A15" s="25" t="n">
-        <x:v>626</x:v>
-      </x:c>
-      <x:c r="B15" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C15" s="25" t="str">
-        <x:v>大霍岭</x:v>
-      </x:c>
-      <x:c r="D15" s="25"/>
-      <x:c r="E15" s="25"/>
-      <x:c r="F15" s="25" t="str">
+      <x:c r="A15" t="n">
+        <x:v>630</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>纯乡</x:v>
+      </x:c>
+      <x:c r="D15"/>
+      <x:c r="E15"/>
+      <x:c r="F15" t="str">
         <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="43.5" customHeight="1">
-      <x:c r="A16" s="25" t="n">
-        <x:v>627</x:v>
-      </x:c>
-      <x:c r="B16" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C16" s="25" t="str">
-        <x:v>龙骨山</x:v>
-      </x:c>
-      <x:c r="D16" s="25"/>
-      <x:c r="E16" s="25"/>
-      <x:c r="F16" s="25" t="str">
-        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；有原始候選，但未同時通過名稱、類型及限制範圍；不得採用其座標。</x:v>
+      <x:c r="A16" t="n">
+        <x:v>631</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>纯乡村</x:v>
+      </x:c>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16" t="str">
+        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="43.5" customHeight="1">
-      <x:c r="A17" s="25" t="n">
-        <x:v>628</x:v>
-      </x:c>
-      <x:c r="B17" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C17" s="25" t="str">
-        <x:v>骨岭</x:v>
-      </x:c>
-      <x:c r="D17" s="25"/>
-      <x:c r="E17" s="25"/>
-      <x:c r="F17" s="25" t="str">
-        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；有原始候選，但未同時通過名稱、類型及限制範圍；不得採用其座標。</x:v>
+      <x:c r="A17" t="n">
+        <x:v>633</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>干冈岭</x:v>
+      </x:c>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17" t="str">
+        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="43.5" customHeight="1">
-      <x:c r="A18" s="25" t="n">
-        <x:v>629</x:v>
-      </x:c>
-      <x:c r="B18" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C18" s="25" t="str">
-        <x:v>幞头岭</x:v>
-      </x:c>
-      <x:c r="D18" s="25"/>
-      <x:c r="E18" s="25"/>
-      <x:c r="F18" s="25" t="str">
+      <x:c r="A18" t="n">
+        <x:v>636</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>巴溪</x:v>
+      </x:c>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18" t="str">
         <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="43.5" customHeight="1">
-      <x:c r="A19" s="25" t="n">
-        <x:v>630</x:v>
-      </x:c>
-      <x:c r="B19" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C19" s="25" t="str">
-        <x:v>纯乡</x:v>
-      </x:c>
-      <x:c r="D19" s="25"/>
-      <x:c r="E19" s="25"/>
-      <x:c r="F19" s="25" t="str">
-        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="43.5" customHeight="1">
-      <x:c r="A20" s="25" t="n">
-        <x:v>631</x:v>
-      </x:c>
-      <x:c r="B20" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C20" s="25" t="str">
-        <x:v>纯乡村</x:v>
-      </x:c>
-      <x:c r="D20" s="25"/>
-      <x:c r="E20" s="25"/>
-      <x:c r="F20" s="25" t="str">
-        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="43.5" customHeight="1">
-      <x:c r="A21" s="25" t="n">
-        <x:v>633</x:v>
-      </x:c>
-      <x:c r="B21" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C21" s="25" t="str">
-        <x:v>干冈岭</x:v>
-      </x:c>
-      <x:c r="D21" s="25"/>
-      <x:c r="E21" s="25"/>
-      <x:c r="F21" s="25" t="str">
-        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="43.5" customHeight="1">
-      <x:c r="A22" s="25" t="n">
-        <x:v>636</x:v>
-      </x:c>
-      <x:c r="B22" s="25" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C22" s="25" t="str">
-        <x:v>巴溪</x:v>
-      </x:c>
-      <x:c r="D22" s="25"/>
-      <x:c r="E22" s="25"/>
-      <x:c r="F22" s="25" t="str">
-        <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="43.5" customHeight="1">
-      <x:c r="A23" s="26" t="n">
+      <x:c r="A19" t="n">
         <x:v>650</x:v>
       </x:c>
-      <x:c r="B23" s="26" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C23" s="26" t="str">
+      <x:c r="B19" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
         <x:v>朱碧街</x:v>
       </x:c>
-      <x:c r="D23" s="26"/>
-      <x:c r="E23" s="26"/>
-      <x:c r="F23" s="26" t="str">
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19" t="str">
         <x:v>未取得可採用座標；查詢來源：CHGIS/TGAZ、OpenStreetMap/Nominatim、Wikidata；Amap／Google Maps僅公開搜尋頁；OSM及Wikidata均無可核驗候選；Amap／Google Maps只保留搜尋連結，未取得可追溯點位。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A2:F2"/>
-    <x:mergeCell ref="A3:F3"/>
-    <x:mergeCell ref="A4:F4"/>
-    <x:mergeCell ref="A5:F5"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R131d4c824af04162"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d5e4992dafa4b1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>